<commit_message>
Re-scoring after BBH newline parsing problem fix
</commit_message>
<xml_diff>
--- a/summaries/summary_report.xlsx
+++ b/summaries/summary_report.xlsx
@@ -1034,7 +1034,7 @@
         <v>10.67</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>44.24</v>
+        <v>46.41</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>6.7</v>
@@ -1055,13 +1055,13 @@
         <v>10.56</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>40.2</v>
+        <v>41.92</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>99.40000000000001</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>40.44</v>
+        <v>42.17</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>0</v>
@@ -1241,7 +1241,7 @@
         <v>100</v>
       </c>
       <c r="BV5" s="6" t="n">
-        <v>0</v>
+        <v>8.65</v>
       </c>
       <c r="BW5" s="6" t="n">
         <v>100</v>
@@ -1288,7 +1288,7 @@
         <v>35.99</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>-1.94</v>
+        <v>-4.11</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>40.62</v>
@@ -1309,13 +1309,13 @@
         <v>11.22</v>
       </c>
       <c r="L6" s="10" t="n">
-        <v>-0.34</v>
+        <v>-2.06</v>
       </c>
       <c r="M6" s="10" t="n">
         <v>-1.6</v>
       </c>
-      <c r="N6" s="9" t="n">
-        <v>0.32</v>
+      <c r="N6" s="10" t="n">
+        <v>-1.41</v>
       </c>
       <c r="O6" s="9" t="n">
         <v>10</v>
@@ -1495,7 +1495,7 @@
         <v>0</v>
       </c>
       <c r="BV6" s="9" t="n">
-        <v>34.62</v>
+        <v>25.97</v>
       </c>
       <c r="BW6" s="11" t="n">
         <v>0</v>
@@ -1542,7 +1542,7 @@
         <v>38.93</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>-0.71</v>
+        <v>-2.88</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>46.42</v>
@@ -1563,13 +1563,13 @@
         <v>15.11</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>-0.68</v>
+        <v>-2.4</v>
       </c>
       <c r="M7" s="9" t="n">
         <v>0.6</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>-0.92</v>
+        <v>-2.65</v>
       </c>
       <c r="O7" s="9" t="n">
         <v>60</v>
@@ -1749,7 +1749,7 @@
         <v>0</v>
       </c>
       <c r="BV7" s="9" t="n">
-        <v>10.58</v>
+        <v>1.93</v>
       </c>
       <c r="BW7" s="11" t="n">
         <v>0</v>
@@ -1795,8 +1795,8 @@
       <c r="D8" s="9" t="n">
         <v>35.34</v>
       </c>
-      <c r="E8" s="9" t="n">
-        <v>0.11</v>
+      <c r="E8" s="10" t="n">
+        <v>-2.06</v>
       </c>
       <c r="F8" s="9" t="n">
         <v>41.54</v>
@@ -1817,13 +1817,13 @@
         <v>18.18</v>
       </c>
       <c r="L8" s="10" t="n">
-        <v>-2.83</v>
+        <v>-4.55</v>
       </c>
       <c r="M8" s="9" t="n">
         <v>0.4</v>
       </c>
       <c r="N8" s="10" t="n">
-        <v>-3</v>
+        <v>-4.73</v>
       </c>
       <c r="O8" s="9" t="n">
         <v>50</v>
@@ -2002,8 +2002,8 @@
       <c r="BU8" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="BV8" s="9" t="n">
-        <v>5.77</v>
+      <c r="BV8" s="10" t="n">
+        <v>-2.88</v>
       </c>
       <c r="BW8" s="11" t="n">
         <v>0</v>
@@ -2050,7 +2050,7 @@
         <v>28.25</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>-0.1</v>
+        <v>-2.27</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>33.54</v>
@@ -2071,13 +2071,13 @@
         <v>13.25</v>
       </c>
       <c r="L9" s="9" t="n">
-        <v>2.73</v>
+        <v>1.01</v>
       </c>
       <c r="M9" s="10" t="n">
         <v>-1.6</v>
       </c>
       <c r="N9" s="9" t="n">
-        <v>3.46</v>
+        <v>1.73</v>
       </c>
       <c r="O9" s="9" t="n">
         <v>100</v>
@@ -2257,7 +2257,7 @@
         <v>0</v>
       </c>
       <c r="BV9" s="9" t="n">
-        <v>39.42</v>
+        <v>30.77</v>
       </c>
       <c r="BW9" s="11" t="n">
         <v>0</v>
@@ -2296,7 +2296,7 @@
         <v>26.66</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>51.33</v>
+        <v>55.08</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>29.28</v>
@@ -2317,13 +2317,13 @@
         <v>39.52</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>48.74</v>
+        <v>53.53</v>
       </c>
       <c r="M10" s="6" t="n">
         <v>99.59999999999999</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>48.94</v>
+        <v>53.74</v>
       </c>
       <c r="O10" s="6" t="n">
         <v>57.5</v>
@@ -2503,7 +2503,7 @@
         <v>100</v>
       </c>
       <c r="BV10" s="6" t="n">
-        <v>0</v>
+        <v>24.04</v>
       </c>
       <c r="BW10" s="6" t="n">
         <v>100</v>
@@ -2549,8 +2549,8 @@
       <c r="D11" s="9" t="n">
         <v>4.92</v>
       </c>
-      <c r="E11" s="9" t="n">
-        <v>2.94</v>
+      <c r="E11" s="10" t="n">
+        <v>-0.8100000000000001</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>4.02</v>
@@ -2570,14 +2570,14 @@
       <c r="K11" s="10" t="n">
         <v>-4.2</v>
       </c>
-      <c r="L11" s="9" t="n">
-        <v>1.58</v>
+      <c r="L11" s="10" t="n">
+        <v>-3.21</v>
       </c>
       <c r="M11" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="N11" s="9" t="n">
-        <v>1.58</v>
+      <c r="N11" s="10" t="n">
+        <v>-3.22</v>
       </c>
       <c r="O11" s="9" t="n">
         <v>17.5</v>
@@ -2756,8 +2756,8 @@
       <c r="BU11" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="BV11" s="9" t="n">
-        <v>20.19</v>
+      <c r="BV11" s="10" t="n">
+        <v>-3.85</v>
       </c>
       <c r="BW11" s="11" t="n">
         <v>0</v>
@@ -2804,7 +2804,7 @@
         <v>-2.39</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>-3.96</v>
+        <v>-7.71</v>
       </c>
       <c r="F12" s="10" t="n">
         <v>-0.8100000000000001</v>
@@ -2825,13 +2825,13 @@
         <v>-20.94</v>
       </c>
       <c r="L12" s="10" t="n">
-        <v>-5.1</v>
+        <v>-9.890000000000001</v>
       </c>
       <c r="M12" s="9" t="n">
         <v>0.2</v>
       </c>
       <c r="N12" s="10" t="n">
-        <v>-5.21</v>
+        <v>-10.01</v>
       </c>
       <c r="O12" s="9" t="n">
         <v>7.5</v>
@@ -3011,7 +3011,7 @@
         <v>0</v>
       </c>
       <c r="BV12" s="9" t="n">
-        <v>30.77</v>
+        <v>6.73</v>
       </c>
       <c r="BW12" s="11" t="n">
         <v>0</v>
@@ -3057,8 +3057,8 @@
       <c r="D13" s="9" t="n">
         <v>6.69</v>
       </c>
-      <c r="E13" s="9" t="n">
-        <v>2.94</v>
+      <c r="E13" s="10" t="n">
+        <v>-0.8100000000000001</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>4.46</v>
@@ -3078,14 +3078,14 @@
       <c r="K13" s="10" t="n">
         <v>-4.2</v>
       </c>
-      <c r="L13" s="9" t="n">
-        <v>1.58</v>
+      <c r="L13" s="10" t="n">
+        <v>-3.21</v>
       </c>
       <c r="M13" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="N13" s="9" t="n">
-        <v>1.58</v>
+      <c r="N13" s="10" t="n">
+        <v>-3.22</v>
       </c>
       <c r="O13" s="9" t="n">
         <v>22.5</v>
@@ -3264,8 +3264,8 @@
       <c r="BU13" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="BV13" s="9" t="n">
-        <v>20.19</v>
+      <c r="BV13" s="10" t="n">
+        <v>-3.85</v>
       </c>
       <c r="BW13" s="11" t="n">
         <v>0</v>
@@ -3550,7 +3550,7 @@
         <v>31.91</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>53.9</v>
+        <v>57.49</v>
       </c>
       <c r="F15" s="6" t="n">
         <v>37.37</v>
@@ -3571,13 +3571,13 @@
         <v>45.07</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>50.2</v>
+        <v>53.85</v>
       </c>
       <c r="M15" s="6" t="n">
         <v>100</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>50.2</v>
+        <v>53.85</v>
       </c>
       <c r="O15" s="6" t="n">
         <v>87.5</v>
@@ -3757,7 +3757,7 @@
         <v>100</v>
       </c>
       <c r="BV15" s="6" t="n">
-        <v>0</v>
+        <v>18.27</v>
       </c>
       <c r="BW15" s="6" t="n">
         <v>100</v>
@@ -3804,7 +3804,7 @@
         <v>4.7</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>-3.98</v>
+        <v>-7.57</v>
       </c>
       <c r="F16" s="9" t="n">
         <v>0.17</v>
@@ -3825,13 +3825,13 @@
         <v>-19.55</v>
       </c>
       <c r="L16" s="10" t="n">
-        <v>-3.44</v>
+        <v>-7.09</v>
       </c>
       <c r="M16" s="10" t="n">
         <v>-0.4</v>
       </c>
       <c r="N16" s="10" t="n">
-        <v>-3.25</v>
+        <v>-6.9</v>
       </c>
       <c r="O16" s="10" t="n">
         <v>-42.5</v>
@@ -4010,8 +4010,8 @@
       <c r="BU16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="BV16" s="9" t="n">
-        <v>1.92</v>
+      <c r="BV16" s="10" t="n">
+        <v>-16.35</v>
       </c>
       <c r="BW16" s="11" t="n">
         <v>0</v>
@@ -4078,14 +4078,14 @@
       <c r="K17" s="10" t="n">
         <v>-0.87</v>
       </c>
-      <c r="L17" s="10" t="n">
-        <v>-0.1</v>
+      <c r="L17" s="9" t="n">
+        <v>0.48</v>
       </c>
       <c r="M17" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="N17" s="10" t="n">
-        <v>-0.1</v>
+      <c r="N17" s="9" t="n">
+        <v>0.48</v>
       </c>
       <c r="O17" s="10" t="n">
         <v>-10</v>
@@ -4264,8 +4264,8 @@
       <c r="BU17" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="BV17" s="11" t="n">
-        <v>0</v>
+      <c r="BV17" s="9" t="n">
+        <v>2.88</v>
       </c>
       <c r="BW17" s="11" t="n">
         <v>0</v>
@@ -4312,7 +4312,7 @@
         <v>21.48</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>3.9</v>
+        <v>0.31</v>
       </c>
       <c r="F18" s="9" t="n">
         <v>22.82</v>
@@ -4333,13 +4333,13 @@
         <v>-8.1</v>
       </c>
       <c r="L18" s="9" t="n">
-        <v>4.29</v>
+        <v>0.64</v>
       </c>
       <c r="M18" s="10" t="n">
         <v>-0.4</v>
       </c>
       <c r="N18" s="9" t="n">
-        <v>4.51</v>
+        <v>0.86</v>
       </c>
       <c r="O18" s="9" t="n">
         <v>12.5</v>
@@ -4519,7 +4519,7 @@
         <v>0</v>
       </c>
       <c r="BV18" s="9" t="n">
-        <v>33.65</v>
+        <v>15.38</v>
       </c>
       <c r="BW18" s="11" t="n">
         <v>0</v>

</xml_diff>